<commit_message>
description sheet formed properly
</commit_message>
<xml_diff>
--- a/far_creation/far.xlsx
+++ b/far_creation/far.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,56 +436,127 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LB IP</t>
+          <t>Node Info</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VIP1 1.1.1.1 
- VIP2 2.2.2.2</t>
+          <t xml:space="preserve"> Bastion/Registry 1.1.1.1
+ Bootstrap 2.2.2.2
+ Master 1 3.3.3.3
+ Master 2 4.4.4.4
+ Worker string
+ Central Bastion 10.177.111.65
+ Central Mirror 10.177.111.66
+</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Vip1 and Vip2</t>
+          <t>Node Ip info</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LDAP url</t>
+          <t>LB IP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ldap-url</t>
+          <t>VIP1: string_vip1
+VIP2: string_vip2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LDAP url</t>
+          <t>VIP info</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Node Info</t>
+          <t>LDAP url</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bastion Nodes: string 
- Bootstrap Nodes: 3.3.3.3, 4.4.4.4 
- Master Nodes: string 
- Worker Nodes: string 
- Infra Nodes: string</t>
+          <t>ldap://something</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Node Ip info</t>
+          <t>This url is used to establish connection between Ocp cluster and vcenter platform as well as authentication</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LDAP IP</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>corp.ad.sbi
+10.189.37.135
+10.189.37.136
+10.189.37.137
+10.176.54.30
+10.176.54.31
+10.176.54.32
+10.176.53.145</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Used for authentication</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NTP IP</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10.191.174.52
+10.191.174.53
+10.179.70.2
+10.179.70.3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Used for time sync</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Windows IP</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10.0.70.28
+10.0.88.137
+10.0.70.26
+10.0.70.17
+10.0.70.239
+10.0.70.23
+10.0.88.148
+10.0.88.151</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Meghdoot OCP Team's desktop IP</t>
         </is>
       </c>
     </row>

</xml_diff>